<commit_message>
add Primary School Expansion cost plan and CVR
</commit_message>
<xml_diff>
--- a/cost-plans/Government-Office-Refurbishment.xlsx
+++ b/cost-plans/Government-Office-Refurbishment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qs\project-cost-control\cost-plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FE76C62-C113-446E-8C65-8DF26DC2019A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18E46400-3EAD-4280-84C3-B429776C1237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" activeTab="1" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost Plan" sheetId="1" r:id="rId1"/>
@@ -506,16 +506,16 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="5" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="37" fontId="1" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="37" fontId="4" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="37" fontId="4" fillId="6" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="37" fontId="1" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="37" fontId="1" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="37" fontId="4" fillId="5" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="37" fontId="4" fillId="6" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="37" fontId="1" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
@@ -524,6 +524,30 @@
     <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="5">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF70AD47"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="0"/>
@@ -541,30 +565,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF70AD47"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2203,7 +2203,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B8CA9C0-9C58-4F75-869D-8D1A35F325AC}">
   <dimension ref="A1:J26"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.6" outlineLevelRow="1" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="12.69140625" style="2" customWidth="1"/>
     <col min="2" max="2" width="35.69140625" customWidth="1"/>
@@ -2216,33 +2216,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
     </row>
     <row r="2" spans="1:10" ht="25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="49" t="str">
+      <c r="A2" s="53" t="str">
         <f ca="1">"Meridian Cost Consultants | Report Date: "&amp;TEXT(TODAY(),"DD MMMM YYYY")</f>
         <v>Meridian Cost Consultants | Report Date: 15 May 2026</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
     </row>
     <row r="4" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="7" t="s">
@@ -2307,7 +2307,7 @@
         <f t="shared" si="0"/>
         <v>545000</v>
       </c>
-      <c r="I5" s="50">
+      <c r="I5" s="48">
         <f>E5-H5</f>
         <v>-20000</v>
       </c>
@@ -2316,7 +2316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A6" s="9" t="s">
         <v>21</v>
       </c>
@@ -2328,7 +2328,7 @@
       </c>
       <c r="D6" s="34"/>
       <c r="E6" s="34">
-        <f t="shared" ref="E6:E26" si="1">C6+D6</f>
+        <f t="shared" ref="E6:E25" si="1">C6+D6</f>
         <v>225000</v>
       </c>
       <c r="F6" s="34">
@@ -2340,7 +2340,7 @@
       <c r="H6" s="34">
         <v>225000</v>
       </c>
-      <c r="I6" s="51">
+      <c r="I6" s="49">
         <f t="shared" ref="I6:I25" si="2">E6-H6</f>
         <v>0</v>
       </c>
@@ -2348,7 +2348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A7" s="10" t="s">
         <v>22</v>
       </c>
@@ -2372,7 +2372,7 @@
       <c r="H7" s="35">
         <v>320000</v>
       </c>
-      <c r="I7" s="52">
+      <c r="I7" s="50">
         <f t="shared" si="2"/>
         <v>-20000</v>
       </c>
@@ -2380,7 +2380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:10" collapsed="1" x14ac:dyDescent="0.4">
       <c r="A8" s="8" t="s">
         <v>23</v>
       </c>
@@ -2411,8 +2411,8 @@
         <f t="shared" si="3"/>
         <v>1120000</v>
       </c>
-      <c r="I8" s="50">
-        <f t="shared" ref="I8" si="4">E8-H8</f>
+      <c r="I8" s="48">
+        <f>E8-H8</f>
         <v>-25000</v>
       </c>
       <c r="J8" s="11">
@@ -2420,7 +2420,7 @@
         <v>0.95479452054794522</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A9" s="9" t="s">
         <v>24</v>
       </c>
@@ -2444,7 +2444,7 @@
       <c r="H9" s="34">
         <v>375000</v>
       </c>
-      <c r="I9" s="51">
+      <c r="I9" s="49">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -2452,7 +2452,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A10" s="10" t="s">
         <v>25</v>
       </c>
@@ -2476,7 +2476,7 @@
       <c r="H10" s="35">
         <v>465000</v>
       </c>
-      <c r="I10" s="52">
+      <c r="I10" s="50">
         <f t="shared" si="2"/>
         <v>-15000</v>
       </c>
@@ -2484,7 +2484,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A11" s="9" t="s">
         <v>26</v>
       </c>
@@ -2510,7 +2510,7 @@
       <c r="H11" s="34">
         <v>280000</v>
       </c>
-      <c r="I11" s="51">
+      <c r="I11" s="49">
         <f t="shared" si="2"/>
         <v>-10000</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:10" collapsed="1" x14ac:dyDescent="0.4">
       <c r="A12" s="8" t="s">
         <v>27</v>
       </c>
@@ -2530,26 +2530,26 @@
         <v>1275000</v>
       </c>
       <c r="D12" s="33">
-        <f t="shared" ref="D12:H12" si="5">SUM(D13:D15)</f>
+        <f t="shared" ref="D12:H12" si="4">SUM(D13:D15)</f>
         <v>0</v>
       </c>
       <c r="E12" s="33">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1275000</v>
       </c>
       <c r="F12" s="33">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1031250</v>
       </c>
       <c r="G12" s="33">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>742500</v>
       </c>
       <c r="H12" s="33">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>1290000</v>
       </c>
-      <c r="I12" s="50">
+      <c r="I12" s="48">
         <f t="shared" si="2"/>
         <v>-15000</v>
       </c>
@@ -2558,7 +2558,7 @@
         <v>0.53529411764705881</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A13" s="9" t="s">
         <v>28</v>
       </c>
@@ -2582,7 +2582,7 @@
       <c r="H13" s="34">
         <v>450000</v>
       </c>
-      <c r="I13" s="51">
+      <c r="I13" s="49">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -2590,7 +2590,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A14" s="10" t="s">
         <v>29</v>
       </c>
@@ -2614,7 +2614,7 @@
       <c r="H14" s="35">
         <v>615000</v>
       </c>
-      <c r="I14" s="52">
+      <c r="I14" s="50">
         <f t="shared" si="2"/>
         <v>-15000</v>
       </c>
@@ -2622,7 +2622,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A15" s="9" t="s">
         <v>53</v>
       </c>
@@ -2646,7 +2646,7 @@
       <c r="H15" s="34">
         <v>225000</v>
       </c>
-      <c r="I15" s="51">
+      <c r="I15" s="49">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:10" collapsed="1" x14ac:dyDescent="0.4">
       <c r="A16" s="8" t="s">
         <v>30</v>
       </c>
@@ -2666,26 +2666,26 @@
         <v>525000</v>
       </c>
       <c r="D16" s="33">
-        <f t="shared" ref="D16:H16" si="6">SUM(D17:D18)</f>
+        <f t="shared" ref="D16:H16" si="5">SUM(D17:D18)</f>
         <v>0</v>
       </c>
       <c r="E16" s="33">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>525000</v>
       </c>
       <c r="F16" s="33">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>292500</v>
       </c>
       <c r="G16" s="33">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>146250</v>
       </c>
       <c r="H16" s="33">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>525000</v>
       </c>
-      <c r="I16" s="50">
+      <c r="I16" s="48">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -2694,7 +2694,7 @@
         <v>0.37857142857142856</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A17" s="9" t="s">
         <v>47</v>
       </c>
@@ -2718,7 +2718,7 @@
       <c r="H17" s="34">
         <v>300000</v>
       </c>
-      <c r="I17" s="51">
+      <c r="I17" s="49">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -2726,7 +2726,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A18" s="10" t="s">
         <v>48</v>
       </c>
@@ -2750,7 +2750,7 @@
       <c r="H18" s="35">
         <v>225000</v>
       </c>
-      <c r="I18" s="52">
+      <c r="I18" s="50">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -2758,7 +2758,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:10" collapsed="1" x14ac:dyDescent="0.4">
       <c r="A19" s="8" t="s">
         <v>31</v>
       </c>
@@ -2770,26 +2770,26 @@
         <v>2700000</v>
       </c>
       <c r="D19" s="33">
-        <f t="shared" ref="D19:H19" si="7">SUM(D20:D22)</f>
+        <f t="shared" ref="D19:H19" si="6">SUM(D20:D22)</f>
         <v>100000</v>
       </c>
       <c r="E19" s="33">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>2800000</v>
       </c>
       <c r="F19" s="33">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>2583500</v>
       </c>
       <c r="G19" s="33">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1872000</v>
       </c>
       <c r="H19" s="33">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>2825000</v>
       </c>
-      <c r="I19" s="50">
+      <c r="I19" s="48">
         <f t="shared" si="2"/>
         <v>-25000</v>
       </c>
@@ -2798,7 +2798,7 @@
         <v>0.61478571428571427</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A20" s="9" t="s">
         <v>32</v>
       </c>
@@ -2824,7 +2824,7 @@
       <c r="H20" s="34">
         <v>1420000</v>
       </c>
-      <c r="I20" s="51">
+      <c r="I20" s="49">
         <f t="shared" si="2"/>
         <v>-2000</v>
       </c>
@@ -2832,7 +2832,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A21" s="10" t="s">
         <v>33</v>
       </c>
@@ -2858,7 +2858,7 @@
       <c r="H21" s="35">
         <v>1095000</v>
       </c>
-      <c r="I21" s="52">
+      <c r="I21" s="50">
         <f t="shared" si="2"/>
         <v>-13000</v>
       </c>
@@ -2866,7 +2866,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:10" hidden="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="A22" s="9" t="s">
         <v>54</v>
       </c>
@@ -2890,7 +2890,7 @@
       <c r="H22" s="34">
         <v>310000</v>
       </c>
-      <c r="I22" s="51">
+      <c r="I22" s="49">
         <f t="shared" si="2"/>
         <v>-10000</v>
       </c>
@@ -2898,7 +2898,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:10" collapsed="1" x14ac:dyDescent="0.4">
       <c r="A23" s="8" t="s">
         <v>34</v>
       </c>
@@ -2922,7 +2922,7 @@
       <c r="H23" s="33">
         <v>225000</v>
       </c>
-      <c r="I23" s="50">
+      <c r="I23" s="48">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -2956,7 +2956,7 @@
       <c r="H24" s="33">
         <v>980000</v>
       </c>
-      <c r="I24" s="50">
+      <c r="I24" s="48">
         <f t="shared" si="2"/>
         <v>-25000</v>
       </c>
@@ -2988,7 +2988,7 @@
       <c r="H25" s="33">
         <v>250000</v>
       </c>
-      <c r="I25" s="50">
+      <c r="I25" s="48">
         <f t="shared" si="2"/>
         <v>50000</v>
       </c>
@@ -3005,15 +3005,15 @@
         <v>7500000</v>
       </c>
       <c r="D26" s="36">
-        <f t="shared" ref="D26:E26" si="8">SUM(D5,D8,D12,D16,D19,D23,D24,D25)</f>
+        <f t="shared" ref="D26:E26" si="7">SUM(D5,D8,D12,D16,D19,D23,D24,D25)</f>
         <v>200000</v>
       </c>
       <c r="E26" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>7700000</v>
       </c>
       <c r="F26" s="36">
-        <f t="shared" ref="F26:H26" si="9">SUM(F5,F8,F12,F16,F19,F23,F24,F25)</f>
+        <f t="shared" ref="F26:H26" si="8">SUM(F5,F8,F12,F16,F19,F23,F24,F25)</f>
         <v>6594750</v>
       </c>
       <c r="G26" s="36">
@@ -3021,10 +3021,10 @@
         <v>4893250</v>
       </c>
       <c r="H26" s="36">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>7760000</v>
       </c>
-      <c r="I26" s="53">
+      <c r="I26" s="51">
         <f>E26-H26</f>
         <v>-60000</v>
       </c>
@@ -3039,20 +3039,20 @@
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <conditionalFormatting sqref="I5:I26">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>AND(I5&lt;0, I5&gt;=-E5*0.02)</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="A5:A25" numberStoredAsText="1"/>
-    <ignoredError sqref="C19 J19" formulaRange="1"/>
+    <ignoredError sqref="C19 J19 F19:H19" formulaRange="1"/>
     <ignoredError sqref="E6:E25" formula="1"/>
   </ignoredErrors>
 </worksheet>
@@ -3071,26 +3071,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="35.049999999999997" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="52" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
     </row>
     <row r="2" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="53" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" s="37" t="s">
@@ -3288,15 +3288,15 @@
         <v>5740000</v>
       </c>
       <c r="D11" s="23">
-        <f t="shared" ref="D11:D23" si="3">B11-C11</f>
+        <f t="shared" ref="D11:D13" si="3">B11-C11</f>
         <v>-220000</v>
       </c>
       <c r="E11" s="17">
-        <f t="shared" ref="E11:E23" si="4">D11/B11</f>
+        <f t="shared" ref="E11:E13" si="4">D11/B11</f>
         <v>-3.9855072463768113E-2</v>
       </c>
       <c r="F11" s="40">
-        <f t="shared" ref="F11:F23" si="5">B11/C11</f>
+        <f t="shared" ref="F11:F13" si="5">B11/C11</f>
         <v>0.9616724738675958</v>
       </c>
       <c r="G11" s="18">
@@ -3464,10 +3464,10 @@
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <conditionalFormatting sqref="D5:D23">
-    <cfRule type="expression" dxfId="4" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>D5&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>D5&lt;0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
add Data Centre Shell and Core cost plan and CVR - all five projects complete
</commit_message>
<xml_diff>
--- a/cost-plans/Government-Office-Refurbishment.xlsx
+++ b/cost-plans/Government-Office-Refurbishment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\qs\project-cost-control\cost-plans\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18E46400-3EAD-4280-84C3-B429776C1237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC3E671-6765-4339-B908-72BD131C29CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14092" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
+    <workbookView xWindow="4714" yWindow="1706" windowWidth="18515" windowHeight="10123" xr2:uid="{0C8C6BE1-598D-4333-9AA5-A074653745B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost Plan" sheetId="1" r:id="rId1"/>

</xml_diff>